<commit_message>
Bid Intelligence v1: embed productivity calibration panel
Inlines OWP_Productivity_Insights.json (50-job benchmark layer)
into index.html as OWP_CALIB constant. New 'Productivity calibration'
section in the Bid Intelligence view between assumptions and the
win-probability curve, rendering:

- 4-tile headline strip: hours/unit (123.4), loaded wage ($40.23),
  gross margin (41.4%), material cushion (-23.9%)
- Cushion code table (5 codes that under-budget consistently)
- Overrun code table (2 codes that over-budget consistently —
  120 Roughin Labor +10.2%, 600 Subcontractor +106%)
- 7 calibration rules (OWP-BID-001..007) with default values,
  P25-P75 bands, rationale, applies-when

Source files committed at owp/bidding tool calibration/ for
regeneration; inline copy is canonical for the dashboard.

Also includes refreshed 2108/2109 JCR + data.json regenerated
by enrichment pass.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/owp/owp-2108-live/cortex output files/OWP_2108_JCR_Cortex_v2.xlsx
+++ b/owp/owp-2108-live/cortex output files/OWP_2108_JCR_Cortex_v2.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="294">
   <si>
     <t xml:space="preserve">OWP #2108 · R&amp;G Apartments</t>
   </si>
@@ -209,6 +209,9 @@
     <t xml:space="preserve">Site Address</t>
   </si>
   <si>
+    <t xml:space="preserve">Seattle, WA — Rainier Ave S × S Genesee St (per AR invoice 'Rainier &amp; Genesee, LLC')</t>
+  </si>
+  <si>
     <t xml:space="preserve">Permit</t>
   </si>
   <si>
@@ -281,10 +284,25 @@
     <t xml:space="preserve">Plumbing Units</t>
   </si>
   <si>
+    <t xml:space="preserve">263  ⚠ UNVERIFIED ESTIMATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Units provenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">⚠ UNVERIFIED ESTIMATE — set by prior session in parse_2108.py PROJECT_META. JDR has no unit count. No GDrive folder mounted. Must be confirmed against drawing P001 or OWP bid sheet once available.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total Fixtures</t>
   </si>
   <si>
-    <t xml:space="preserve">TBD (no fixture schedule yet)</t>
+    <t xml:space="preserve">UNKNOWN  ⚠ no fixture schedule available</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixtures provenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNKNOWN — no fixture schedule available (pre-construction · no design drawings extracted yet).</t>
   </si>
   <si>
     <t xml:space="preserve">Floors</t>
@@ -323,9 +341,15 @@
     <t xml:space="preserve">Owner of Record</t>
   </si>
   <si>
+    <t xml:space="preserve">Lake Union Partners (per AR invoice 'Lake Union Partners $R&amp;G Apts')</t>
+  </si>
+  <si>
     <t xml:space="preserve">Developer</t>
   </si>
   <si>
+    <t xml:space="preserve">Lake Union Partners (per AR billing)</t>
+  </si>
+  <si>
     <t xml:space="preserve">PROJECT TEAM — DESIGN</t>
   </si>
   <si>
@@ -888,6 +912,12 @@
   </si>
   <si>
     <t xml:space="preserve">Enriched Job Info tab with 11-section sectioned layout (identity / schedule / financial posture / scope / project team — 4 sub-sections / document meta / data sources / risk flags). Corrected status from 'CANCELLED' (template default) to 'ON HOLD · Summer 2026?'. Predictive Signals expanded with pre-construction-specific signals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v1.2 · units audit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audited unit/fixture counts. Units 263 flagged as UNVERIFIED ESTIMATE (no source-doc verification possible — JDR has no unit count, no GDrive folder mounted). Fixtures marked UNKNOWN. Recovered owner from JDR AR section: Lake Union Partners. Recovered location: Rainier &amp; Genesee intersection (Columbia City, Seattle).</t>
   </si>
 </sst>
 </file>
@@ -1075,14 +1105,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD4EDDA"/>
-        <bgColor rgb="FFD1ECF1"/>
+        <fgColor rgb="FFFFF3CD"/>
+        <bgColor rgb="FFFFF8E7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF3CD"/>
-        <bgColor rgb="FFFFF8E7"/>
+        <fgColor rgb="FFD4EDDA"/>
+        <bgColor rgb="FFD1ECF1"/>
       </patternFill>
     </fill>
     <fill>
@@ -1092,7 +1122,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1129,6 +1159,17 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD5D8DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD5D8DC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
         <color rgb="FFBFB8AE"/>
       </left>
@@ -1169,7 +1210,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="53">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1214,23 +1255,19 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1242,11 +1279,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1262,11 +1295,27 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1274,12 +1323,12 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1326,6 +1375,10 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1338,19 +1391,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1358,16 +1407,20 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1771,7 +1824,7 @@
         <v>-91402</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
         <v>20</v>
       </c>
@@ -1781,361 +1834,242 @@
       <c r="E40" s="11"/>
       <c r="F40" s="11"/>
       <c r="G40" s="11"/>
-      <c r="H40" s="12"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
+      <c r="H40" s="1"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
-      <c r="H41" s="12"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12"/>
-      <c r="B42" s="12"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="12"/>
-      <c r="F42" s="12"/>
-      <c r="G42" s="12"/>
-      <c r="H42" s="12"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14" t="s">
+      <c r="B41" s="12"/>
+      <c r="C41" s="12"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="12"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B43" s="14" t="s">
+      <c r="B43" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C43" s="12"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="12"/>
-      <c r="F43" s="12"/>
-      <c r="G43" s="12"/>
-      <c r="H43" s="12"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15" t="s">
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B44" s="16" t="s">
+      <c r="B44" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C44" s="12"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="12"/>
-      <c r="G44" s="12"/>
-      <c r="H44" s="12"/>
-    </row>
-    <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="15" t="s">
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+    </row>
+    <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B45" s="16" t="s">
+      <c r="B45" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="12"/>
-      <c r="G45" s="12"/>
-      <c r="H45" s="12"/>
-    </row>
-    <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="15" t="s">
+      <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+    </row>
+    <row r="46" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B46" s="16" t="s">
+      <c r="B46" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="12"/>
-      <c r="F46" s="12"/>
-      <c r="G46" s="12"/>
-      <c r="H46" s="12"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15" t="s">
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B47" s="16" t="s">
+      <c r="B47" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="12"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="s">
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B48" s="16" t="s">
+      <c r="B48" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
-      <c r="F48" s="12"/>
-      <c r="G48" s="12"/>
-      <c r="H48" s="12"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="s">
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B49" s="16" t="s">
+      <c r="B49" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C49" s="12"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="12"/>
-      <c r="F49" s="12"/>
-      <c r="G49" s="12"/>
-      <c r="H49" s="12"/>
-    </row>
-    <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15" t="s">
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+    </row>
+    <row r="50" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B50" s="16" t="s">
+      <c r="B50" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="C50" s="12"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="12"/>
-      <c r="F50" s="12"/>
-      <c r="G50" s="12"/>
-      <c r="H50" s="12"/>
-    </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="15" t="s">
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+    </row>
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B51" s="16" t="s">
+      <c r="B51" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C51" s="12"/>
-      <c r="D51" s="12"/>
-      <c r="E51" s="12"/>
-      <c r="F51" s="12"/>
-      <c r="G51" s="12"/>
-      <c r="H51" s="12"/>
-    </row>
-    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="15" t="s">
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+    </row>
+    <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="B52" s="16" t="s">
+      <c r="B52" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C52" s="12"/>
-      <c r="D52" s="12"/>
-      <c r="E52" s="12"/>
-      <c r="F52" s="12"/>
-      <c r="G52" s="12"/>
-      <c r="H52" s="12"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="15" t="s">
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="B53" s="16" t="s">
+      <c r="B53" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C53" s="12"/>
-      <c r="D53" s="12"/>
-      <c r="E53" s="12"/>
-      <c r="F53" s="12"/>
-      <c r="G53" s="12"/>
-      <c r="H53" s="12"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="15" t="s">
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B54" s="16" t="s">
+      <c r="B54" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="C54" s="12"/>
-      <c r="D54" s="12"/>
-      <c r="E54" s="12"/>
-      <c r="F54" s="12"/>
-      <c r="G54" s="12"/>
-      <c r="H54" s="12"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="15" t="s">
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B55" s="16" t="s">
+      <c r="B55" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="C55" s="12"/>
-      <c r="D55" s="12"/>
-      <c r="E55" s="12"/>
-      <c r="F55" s="12"/>
-      <c r="G55" s="12"/>
-      <c r="H55" s="12"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="12"/>
-      <c r="B56" s="12"/>
-      <c r="C56" s="12"/>
-      <c r="D56" s="12"/>
-      <c r="E56" s="12"/>
-      <c r="F56" s="12"/>
-      <c r="G56" s="12"/>
-      <c r="H56" s="12"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="12"/>
-      <c r="B57" s="12"/>
-      <c r="C57" s="12"/>
-      <c r="D57" s="12"/>
-      <c r="E57" s="12"/>
-      <c r="F57" s="12"/>
-      <c r="G57" s="12"/>
-      <c r="H57" s="12"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="12"/>
-      <c r="B58" s="12"/>
-      <c r="C58" s="12"/>
-      <c r="D58" s="12"/>
-      <c r="E58" s="12"/>
-      <c r="F58" s="12"/>
-      <c r="G58" s="12"/>
-      <c r="H58" s="12"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="12"/>
-      <c r="B59" s="12"/>
-      <c r="C59" s="12"/>
-      <c r="D59" s="12"/>
-      <c r="E59" s="12"/>
-      <c r="F59" s="12"/>
-      <c r="G59" s="12"/>
-      <c r="H59" s="12"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="12"/>
-      <c r="B60" s="12"/>
-      <c r="C60" s="12"/>
-      <c r="D60" s="12"/>
-      <c r="E60" s="12"/>
-      <c r="F60" s="12"/>
-      <c r="G60" s="12"/>
-      <c r="H60" s="12"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="12"/>
-      <c r="B61" s="12"/>
-      <c r="C61" s="12"/>
-      <c r="D61" s="12"/>
-      <c r="E61" s="12"/>
-      <c r="F61" s="12"/>
-      <c r="G61" s="12"/>
-      <c r="H61" s="12"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="12"/>
-      <c r="B62" s="12"/>
-      <c r="C62" s="12"/>
-      <c r="D62" s="12"/>
-      <c r="E62" s="12"/>
-      <c r="F62" s="12"/>
-      <c r="G62" s="12"/>
-      <c r="H62" s="12"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="12"/>
-      <c r="B63" s="12"/>
-      <c r="C63" s="12"/>
-      <c r="D63" s="12"/>
-      <c r="E63" s="12"/>
-      <c r="F63" s="12"/>
-      <c r="G63" s="12"/>
-      <c r="H63" s="12"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="12"/>
-      <c r="B64" s="12"/>
-      <c r="C64" s="12"/>
-      <c r="D64" s="12"/>
-      <c r="E64" s="12"/>
-      <c r="F64" s="12"/>
-      <c r="G64" s="12"/>
-      <c r="H64" s="12"/>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="12"/>
-      <c r="B65" s="12"/>
-      <c r="C65" s="12"/>
-      <c r="D65" s="12"/>
-      <c r="E65" s="12"/>
-      <c r="F65" s="12"/>
-      <c r="G65" s="12"/>
-      <c r="H65" s="12"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="12"/>
-      <c r="B66" s="12"/>
-      <c r="C66" s="12"/>
-      <c r="D66" s="12"/>
-      <c r="E66" s="12"/>
-      <c r="F66" s="12"/>
-      <c r="G66" s="12"/>
-      <c r="H66" s="12"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="12"/>
-      <c r="B67" s="12"/>
-      <c r="C67" s="12"/>
-      <c r="D67" s="12"/>
-      <c r="E67" s="12"/>
-      <c r="F67" s="12"/>
-      <c r="G67" s="12"/>
-      <c r="H67" s="12"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="12"/>
-      <c r="B68" s="12"/>
-      <c r="C68" s="12"/>
-      <c r="D68" s="12"/>
-      <c r="E68" s="12"/>
-      <c r="F68" s="12"/>
-      <c r="G68" s="12"/>
-      <c r="H68" s="12"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="12"/>
-      <c r="B69" s="12"/>
-      <c r="C69" s="12"/>
-      <c r="D69" s="12"/>
-      <c r="E69" s="12"/>
-      <c r="F69" s="12"/>
-      <c r="G69" s="12"/>
-      <c r="H69" s="12"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="12"/>
-      <c r="B70" s="12"/>
-      <c r="C70" s="12"/>
-      <c r="D70" s="12"/>
-      <c r="E70" s="12"/>
-      <c r="F70" s="12"/>
-      <c r="G70" s="12"/>
-      <c r="H70" s="12"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
+      <c r="H61" s="1"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="H62" s="1"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F64" s="1"/>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F65" s="1"/>
+      <c r="G65" s="1"/>
+      <c r="H65" s="1"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F66" s="1"/>
+      <c r="G66" s="1"/>
+      <c r="H66" s="1"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F67" s="1"/>
+      <c r="G67" s="1"/>
+      <c r="H67" s="1"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F68" s="1"/>
+      <c r="G68" s="1"/>
+      <c r="H68" s="1"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2168,60 +2102,60 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>194</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>195</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>196</v>
-      </c>
-      <c r="E3" s="26" t="s">
-        <v>197</v>
+      <c r="A3" s="29" t="s">
+        <v>201</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>203</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>204</v>
+      </c>
+      <c r="E3" s="29" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="B4" s="33" t="n">
+        <v>206</v>
+      </c>
+      <c r="B4" s="35" t="n">
         <v>20.5</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>1414</v>
       </c>
-      <c r="D4" s="34" t="n">
+      <c r="D4" s="36" t="n">
         <f aca="false">IFERROR(C4/B4,0)</f>
         <v>68.9756097560976</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="B5" s="33" t="n">
+        <v>208</v>
+      </c>
+      <c r="B5" s="35" t="n">
         <v>12</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>720</v>
       </c>
-      <c r="D5" s="34" t="n">
+      <c r="D5" s="36" t="n">
         <f aca="false">IFERROR(C5/B5,0)</f>
         <v>60</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -2251,94 +2185,94 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>197</v>
-      </c>
-      <c r="B3" s="26" t="s">
+      <c r="A3" s="29" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="C3" s="29" t="s">
         <v>202</v>
       </c>
-      <c r="C3" s="26" t="s">
-        <v>194</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>195</v>
-      </c>
-      <c r="E3" s="26" t="s">
+      <c r="D3" s="29" t="s">
         <v>203</v>
       </c>
+      <c r="E3" s="29" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>199</v>
+      <c r="A4" s="17" t="s">
+        <v>207</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="33" t="n">
+      <c r="C4" s="35" t="n">
         <v>32.5</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>2134</v>
       </c>
-      <c r="E4" s="28" t="n">
+      <c r="E4" s="30" t="n">
         <f aca="false">IFERROR(C4/SUM(C$4:C$7),0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="s">
-        <v>204</v>
+      <c r="A5" s="17" t="s">
+        <v>212</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="33" t="n">
+      <c r="C5" s="35" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="28" t="n">
+      <c r="E5" s="30" t="n">
         <f aca="false">IFERROR(C5/SUM(C$4:C$7),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="27" t="s">
-        <v>205</v>
+      <c r="A6" s="17" t="s">
+        <v>213</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="33" t="n">
+      <c r="C6" s="35" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="28" t="n">
+      <c r="E6" s="30" t="n">
         <f aca="false">IFERROR(C6/SUM(C$4:C$7),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="27" t="s">
-        <v>206</v>
+      <c r="A7" s="17" t="s">
+        <v>214</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="33" t="n">
+      <c r="C7" s="35" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="28" t="n">
+      <c r="E7" s="30" t="n">
         <f aca="false">IFERROR(C7/SUM(C$4:C$7),0)</f>
         <v>0</v>
       </c>
@@ -2368,38 +2302,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B3" s="33" t="n">
+        <v>216</v>
+      </c>
+      <c r="B3" s="35" t="n">
         <v>32</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="B4" s="35" t="n">
+        <v>217</v>
+      </c>
+      <c r="B4" s="37" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="B5" s="33" t="n">
+        <v>218</v>
+      </c>
+      <c r="B5" s="35" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="B6" s="36" t="n">
+        <v>219</v>
+      </c>
+      <c r="B6" s="38" t="n">
         <v>2812.37</v>
       </c>
     </row>
@@ -2407,7 +2341,7 @@
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2436,79 +2370,79 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>213</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>214</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>215</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>134</v>
+      <c r="A3" s="29" t="s">
+        <v>221</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>222</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>223</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="B4" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="37" t="n">
+        <v>224</v>
+      </c>
+      <c r="B4" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="39" t="n">
         <v>0.34</v>
       </c>
-      <c r="D4" s="28" t="n">
+      <c r="D4" s="30" t="n">
         <f aca="false">B4-C4</f>
         <v>-0.34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="B5" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="37" t="n">
+        <v>225</v>
+      </c>
+      <c r="B5" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="39" t="n">
         <v>0.45</v>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="30" t="n">
         <f aca="false">B5-C5</f>
         <v>-0.45</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="B6" s="37" t="n">
+        <v>226</v>
+      </c>
+      <c r="B6" s="39" t="n">
         <v>0.925225949969935</v>
       </c>
-      <c r="C6" s="37" t="n">
+      <c r="C6" s="39" t="n">
         <v>0.38</v>
       </c>
-      <c r="D6" s="28" t="n">
+      <c r="D6" s="30" t="n">
         <f aca="false">B6-C6</f>
         <v>0.545225949969935</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="B7" s="33" t="n">
+        <v>227</v>
+      </c>
+      <c r="B7" s="35" t="n">
         <v>0.123574144486692</v>
       </c>
-      <c r="C7" s="33" t="n">
+      <c r="C7" s="35" t="n">
         <v>95</v>
       </c>
-      <c r="D7" s="38" t="n">
+      <c r="D7" s="40" t="n">
         <f aca="false">B7-C7</f>
         <v>-94.8764258555133</v>
       </c>
@@ -2535,361 +2469,267 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>220</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
+      <c r="A1" s="41" t="s">
+        <v>228</v>
+      </c>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="39" t="s">
-        <v>151</v>
-      </c>
-      <c r="B3" s="39" t="s">
-        <v>221</v>
-      </c>
-      <c r="C3" s="39" t="s">
-        <v>222</v>
-      </c>
-      <c r="D3" s="39" t="s">
-        <v>223</v>
-      </c>
-      <c r="E3" s="39" t="s">
-        <v>224</v>
-      </c>
-      <c r="F3" s="12"/>
+      <c r="A3" s="42" t="s">
+        <v>159</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>229</v>
+      </c>
+      <c r="C3" s="42" t="s">
+        <v>230</v>
+      </c>
+      <c r="D3" s="42" t="s">
+        <v>231</v>
+      </c>
+      <c r="E3" s="42" t="s">
+        <v>232</v>
+      </c>
+      <c r="F3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="40" t="n">
+      <c r="A4" s="43" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="41" t="s">
-        <v>225</v>
-      </c>
-      <c r="C4" s="40" t="s">
-        <v>226</v>
-      </c>
-      <c r="D4" s="42" t="s">
-        <v>227</v>
-      </c>
-      <c r="E4" s="43" t="s">
-        <v>228</v>
-      </c>
-      <c r="F4" s="12"/>
+      <c r="B4" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="C4" s="43" t="s">
+        <v>234</v>
+      </c>
+      <c r="D4" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="E4" s="45" t="s">
+        <v>236</v>
+      </c>
+      <c r="F4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="40" t="n">
+      <c r="A5" s="43" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="41" t="s">
-        <v>229</v>
-      </c>
-      <c r="C5" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="D5" s="42" t="s">
-        <v>230</v>
-      </c>
-      <c r="E5" s="43" t="s">
-        <v>228</v>
-      </c>
-      <c r="F5" s="12"/>
+      <c r="B5" s="44" t="s">
+        <v>237</v>
+      </c>
+      <c r="C5" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" s="43" t="s">
+        <v>238</v>
+      </c>
+      <c r="E5" s="45" t="s">
+        <v>236</v>
+      </c>
+      <c r="F5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="40" t="n">
+      <c r="A6" s="43" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="41" t="s">
-        <v>231</v>
-      </c>
-      <c r="C6" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="D6" s="42" t="s">
-        <v>232</v>
-      </c>
-      <c r="E6" s="43" t="s">
-        <v>228</v>
-      </c>
-      <c r="F6" s="12"/>
+      <c r="B6" s="44" t="s">
+        <v>239</v>
+      </c>
+      <c r="C6" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="E6" s="45" t="s">
+        <v>236</v>
+      </c>
+      <c r="F6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="40" t="n">
+      <c r="A7" s="43" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="41" t="s">
-        <v>147</v>
-      </c>
-      <c r="C7" s="40" t="s">
-        <v>233</v>
-      </c>
-      <c r="D7" s="42" t="s">
-        <v>234</v>
-      </c>
-      <c r="E7" s="43" t="s">
-        <v>228</v>
-      </c>
-      <c r="F7" s="12"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="42" t="n">
+      <c r="B7" s="44" t="s">
+        <v>155</v>
+      </c>
+      <c r="C7" s="43" t="s">
+        <v>241</v>
+      </c>
+      <c r="D7" s="43" t="s">
+        <v>242</v>
+      </c>
+      <c r="E7" s="45" t="s">
+        <v>236</v>
+      </c>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="43" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="42" t="s">
-        <v>235</v>
-      </c>
-      <c r="C8" s="42" t="s">
-        <v>236</v>
-      </c>
-      <c r="D8" s="42" t="s">
-        <v>237</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>238</v>
-      </c>
-      <c r="F8" s="12"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="42" t="n">
+      <c r="B8" s="43" t="s">
+        <v>243</v>
+      </c>
+      <c r="C8" s="43" t="s">
+        <v>244</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>245</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="43" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="42" t="s">
-        <v>239</v>
-      </c>
-      <c r="C9" s="42" t="s">
+      <c r="B9" s="43" t="s">
+        <v>247</v>
+      </c>
+      <c r="C9" s="43" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="42" t="s">
-        <v>240</v>
-      </c>
-      <c r="E9" s="44" t="s">
+      <c r="D9" s="43" t="s">
+        <v>248</v>
+      </c>
+      <c r="E9" s="46" t="s">
+        <v>249</v>
+      </c>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="43" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="43" t="s">
+        <v>250</v>
+      </c>
+      <c r="C10" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="43" t="s">
         <v>241</v>
       </c>
-      <c r="F9" s="12"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="42" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="42" t="s">
-        <v>242</v>
-      </c>
-      <c r="C10" s="42" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="42" t="s">
-        <v>233</v>
-      </c>
-      <c r="E10" s="44" t="s">
-        <v>241</v>
-      </c>
-      <c r="F10" s="12"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="42" t="n">
+      <c r="E10" s="46" t="s">
+        <v>249</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="43" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="42" t="s">
-        <v>243</v>
-      </c>
-      <c r="C11" s="42" t="s">
+      <c r="B11" s="43" t="s">
+        <v>251</v>
+      </c>
+      <c r="C11" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="42" t="s">
-        <v>244</v>
-      </c>
-      <c r="E11" s="45" t="s">
-        <v>245</v>
-      </c>
-      <c r="F11" s="12"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="42" t="n">
+      <c r="D11" s="43" t="s">
+        <v>252</v>
+      </c>
+      <c r="E11" s="47" t="s">
+        <v>253</v>
+      </c>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="43" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="42" t="s">
-        <v>246</v>
-      </c>
-      <c r="C12" s="42" t="s">
-        <v>102</v>
-      </c>
-      <c r="D12" s="42" t="s">
-        <v>247</v>
-      </c>
-      <c r="E12" s="45" t="s">
-        <v>245</v>
-      </c>
-      <c r="F12" s="12"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="42" t="n">
+      <c r="B12" s="43" t="s">
+        <v>254</v>
+      </c>
+      <c r="C12" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12" s="43" t="s">
+        <v>255</v>
+      </c>
+      <c r="E12" s="47" t="s">
+        <v>253</v>
+      </c>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="43" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="42" t="s">
-        <v>248</v>
-      </c>
-      <c r="C13" s="42" t="s">
+      <c r="B13" s="43" t="s">
+        <v>256</v>
+      </c>
+      <c r="C13" s="43" t="s">
+        <v>257</v>
+      </c>
+      <c r="D13" s="43" t="s">
+        <v>255</v>
+      </c>
+      <c r="E13" s="46" t="s">
         <v>249</v>
       </c>
-      <c r="D13" s="42" t="s">
-        <v>247</v>
-      </c>
-      <c r="E13" s="44" t="s">
-        <v>241</v>
-      </c>
-      <c r="F13" s="12"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F14" s="1"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F18" s="1"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F30" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2916,26 +2756,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="26" t="s">
-        <v>251</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>252</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>134</v>
+      <c r="B3" s="29" t="s">
+        <v>259</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>260</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="B4" s="6" t="n">
         <v>117161.97</v>
@@ -2950,7 +2790,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="B5" s="6" t="n">
         <v>-91402</v>
@@ -2965,7 +2805,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>97953.1</v>
@@ -2977,7 +2817,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>3350.12</v>
@@ -2989,7 +2829,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>15858.75</v>
@@ -3025,84 +2865,84 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>213</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>259</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>260</v>
+      <c r="A3" s="29" t="s">
+        <v>221</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>267</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="46" t="s">
-        <v>216</v>
-      </c>
-      <c r="B4" s="46" t="s">
-        <v>261</v>
-      </c>
-      <c r="C4" s="46" t="s">
-        <v>262</v>
+      <c r="A4" s="48" t="s">
+        <v>224</v>
+      </c>
+      <c r="B4" s="48" t="s">
+        <v>269</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="46" t="s">
-        <v>261</v>
-      </c>
-      <c r="C5" s="46" t="s">
-        <v>263</v>
+      <c r="B5" s="48" t="s">
+        <v>269</v>
+      </c>
+      <c r="C5" s="48" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="46" t="s">
-        <v>264</v>
-      </c>
-      <c r="B6" s="46" t="s">
-        <v>265</v>
-      </c>
-      <c r="C6" s="46" t="s">
-        <v>266</v>
+      <c r="A6" s="48" t="s">
+        <v>272</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>273</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="46" t="s">
-        <v>218</v>
-      </c>
-      <c r="B7" s="46" t="s">
-        <v>267</v>
-      </c>
-      <c r="C7" s="46" t="s">
-        <v>268</v>
+      <c r="A7" s="48" t="s">
+        <v>226</v>
+      </c>
+      <c r="B7" s="48" t="s">
+        <v>275</v>
+      </c>
+      <c r="C7" s="48" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="46" t="s">
-        <v>219</v>
-      </c>
-      <c r="B8" s="46" t="s">
-        <v>269</v>
-      </c>
-      <c r="C8" s="46" t="s">
-        <v>270</v>
+      <c r="A8" s="48" t="s">
+        <v>227</v>
+      </c>
+      <c r="B8" s="48" t="s">
+        <v>277</v>
+      </c>
+      <c r="C8" s="48" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="46" t="s">
-        <v>271</v>
-      </c>
-      <c r="B9" s="46" t="s">
-        <v>272</v>
-      </c>
-      <c r="C9" s="46" t="s">
-        <v>273</v>
+      <c r="A9" s="48" t="s">
+        <v>279</v>
+      </c>
+      <c r="B9" s="48" t="s">
+        <v>280</v>
+      </c>
+      <c r="C9" s="48" t="s">
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -3121,7 +2961,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
@@ -3131,40 +2971,51 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>275</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>276</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>277</v>
+      <c r="A3" s="29" t="s">
+        <v>283</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>284</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="47" t="s">
-        <v>281</v>
-      </c>
-      <c r="B5" s="48" t="s">
-        <v>282</v>
-      </c>
-      <c r="C5" s="49" t="s">
-        <v>283</v>
+        <v>288</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="49" t="s">
+        <v>289</v>
+      </c>
+      <c r="B5" s="50" t="s">
+        <v>290</v>
+      </c>
+      <c r="C5" s="51" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="52" t="s">
+        <v>289</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>292</v>
+      </c>
+      <c r="C6" s="51" t="s">
+        <v>293</v>
       </c>
     </row>
   </sheetData>
@@ -3183,828 +3034,886 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
+      <c r="A3" s="17"/>
+      <c r="B3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17"/>
+      <c r="B11" s="5"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="B14" s="22" t="s">
-        <v>63</v>
-      </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="22" t="s">
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+    </row>
+    <row r="32" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="B32" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+    </row>
+    <row r="34" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="B34" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="B35" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="B19" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="s">
-        <v>70</v>
-      </c>
-      <c r="B20" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="B22" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="B24" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="B26" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="B27" s="22" t="s">
-        <v>76</v>
-      </c>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="B28" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="B31" s="22" t="n">
-        <v>263</v>
-      </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="B32" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="B33" s="22" t="s">
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="B36" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="B34" s="22" t="s">
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="26"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="26"/>
+      <c r="F37" s="26"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B39" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C39" s="27"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="27"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B40" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B41" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="B36" s="24"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="B37" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="C37" s="25"/>
-      <c r="D37" s="25"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="B38" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="C38" s="25"/>
-      <c r="D38" s="25"/>
-      <c r="E38" s="25"/>
-      <c r="F38" s="25"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="B39" s="25" t="s">
+      <c r="C41" s="24"/>
+      <c r="D41" s="24"/>
+      <c r="E41" s="24"/>
+      <c r="F41" s="24"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="B42" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="C39" s="25"/>
-      <c r="D39" s="25"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="B40" s="25" t="s">
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B43" s="26"/>
+      <c r="C43" s="26"/>
+      <c r="D43" s="26"/>
+      <c r="E43" s="26"/>
+      <c r="F43" s="26"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B44" s="24"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B45" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="C45" s="27"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="27"/>
+      <c r="F45" s="27"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B46" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C40" s="25"/>
-      <c r="D40" s="25"/>
-      <c r="E40" s="25"/>
-      <c r="F40" s="25"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="B42" s="24"/>
-      <c r="C42" s="24"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="24"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="B43" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="C43" s="25"/>
-      <c r="D43" s="25"/>
-      <c r="E43" s="25"/>
-      <c r="F43" s="25"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="B44" s="25" t="s">
+      <c r="C46" s="27"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="F46" s="27"/>
+    </row>
+    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B47" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="C47" s="24"/>
+      <c r="D47" s="24"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B48" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="28"/>
+      <c r="F48" s="28"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B49" s="26"/>
+      <c r="C49" s="26"/>
+      <c r="D49" s="26"/>
+      <c r="E49" s="26"/>
+      <c r="F49" s="26"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="B50" s="24"/>
+      <c r="C50" s="24"/>
+      <c r="D50" s="24"/>
+      <c r="E50" s="24"/>
+      <c r="F50" s="24"/>
+    </row>
+    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B51" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C51" s="24"/>
+      <c r="D51" s="24"/>
+      <c r="E51" s="24"/>
+      <c r="F51" s="24"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B52" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="C52" s="28"/>
+      <c r="D52" s="28"/>
+      <c r="E52" s="28"/>
+      <c r="F52" s="28"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B53" s="26"/>
+      <c r="C53" s="26"/>
+      <c r="D53" s="26"/>
+      <c r="E53" s="26"/>
+      <c r="F53" s="26"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B54" s="24"/>
+      <c r="C54" s="24"/>
+      <c r="D54" s="24"/>
+      <c r="E54" s="24"/>
+      <c r="F54" s="24"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B55" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C44" s="25"/>
-      <c r="D44" s="25"/>
-      <c r="E44" s="25"/>
-      <c r="F44" s="25"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="B45" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="C45" s="25"/>
-      <c r="D45" s="25"/>
-      <c r="E45" s="25"/>
-      <c r="F45" s="25"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B46" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="C46" s="25"/>
-      <c r="D46" s="25"/>
-      <c r="E46" s="25"/>
-      <c r="F46" s="25"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="24" t="s">
-        <v>93</v>
-      </c>
-      <c r="B48" s="24"/>
-      <c r="C48" s="24"/>
-      <c r="D48" s="24"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="24"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="B49" s="25" t="s">
+      <c r="C55" s="27"/>
+      <c r="D55" s="27"/>
+      <c r="E55" s="27"/>
+      <c r="F55" s="27"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B56" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C49" s="25"/>
-      <c r="D49" s="25"/>
-      <c r="E49" s="25"/>
-      <c r="F49" s="25"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="B50" s="25" t="s">
+      <c r="C56" s="27"/>
+      <c r="D56" s="27"/>
+      <c r="E56" s="27"/>
+      <c r="F56" s="27"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B57" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C57" s="27"/>
+      <c r="D57" s="27"/>
+      <c r="E57" s="27"/>
+      <c r="F57" s="27"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B58" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C50" s="25"/>
-      <c r="D50" s="25"/>
-      <c r="E50" s="25"/>
-      <c r="F50" s="25"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="B52" s="24"/>
-      <c r="C52" s="24"/>
-      <c r="D52" s="24"/>
-      <c r="E52" s="24"/>
-      <c r="F52" s="24"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="B53" s="25" t="s">
+      <c r="C58" s="24"/>
+      <c r="D58" s="24"/>
+      <c r="E58" s="24"/>
+      <c r="F58" s="24"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="B59" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="C53" s="25"/>
-      <c r="D53" s="25"/>
-      <c r="E53" s="25"/>
-      <c r="F53" s="25"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="B54" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="C54" s="25"/>
-      <c r="D54" s="25"/>
-      <c r="E54" s="25"/>
-      <c r="F54" s="25"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="B55" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C55" s="25"/>
-      <c r="D55" s="25"/>
-      <c r="E55" s="25"/>
-      <c r="F55" s="25"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="B56" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="C56" s="25"/>
-      <c r="D56" s="25"/>
-      <c r="E56" s="25"/>
-      <c r="F56" s="25"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="B57" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="C57" s="25"/>
-      <c r="D57" s="25"/>
-      <c r="E57" s="25"/>
-      <c r="F57" s="25"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="24" t="s">
-        <v>100</v>
-      </c>
-      <c r="B59" s="24"/>
-      <c r="C59" s="24"/>
-      <c r="D59" s="24"/>
-      <c r="E59" s="24"/>
-      <c r="F59" s="24"/>
+      <c r="C59" s="28"/>
+      <c r="D59" s="28"/>
+      <c r="E59" s="28"/>
+      <c r="F59" s="28"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="B60" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C60" s="22"/>
-      <c r="D60" s="22"/>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
+      <c r="B60" s="26"/>
+      <c r="C60" s="26"/>
+      <c r="D60" s="26"/>
+      <c r="E60" s="26"/>
+      <c r="F60" s="26"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="B61" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C61" s="22"/>
-      <c r="D61" s="22"/>
-      <c r="E61" s="22"/>
-      <c r="F61" s="22"/>
+      <c r="A61" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B61" s="24"/>
+      <c r="C61" s="24"/>
+      <c r="D61" s="24"/>
+      <c r="E61" s="24"/>
+      <c r="F61" s="24"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="B62" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C62" s="22"/>
-      <c r="D62" s="22"/>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
+      <c r="A62" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="20"/>
+      <c r="D62" s="20"/>
+      <c r="E62" s="20"/>
+      <c r="F62" s="20"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="23" t="s">
-        <v>105</v>
-      </c>
-      <c r="B63" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C63" s="22"/>
-      <c r="D63" s="22"/>
-      <c r="E63" s="22"/>
-      <c r="F63" s="22"/>
+      <c r="A63" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="B63" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C63" s="20"/>
+      <c r="D63" s="20"/>
+      <c r="E63" s="20"/>
+      <c r="F63" s="20"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="B64" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C64" s="22"/>
-      <c r="D64" s="22"/>
-      <c r="E64" s="22"/>
-      <c r="F64" s="22"/>
+      <c r="A64" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="B64" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C64" s="20"/>
+      <c r="D64" s="20"/>
+      <c r="E64" s="20"/>
+      <c r="F64" s="20"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="B65" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C65" s="22"/>
-      <c r="D65" s="22"/>
-      <c r="E65" s="22"/>
-      <c r="F65" s="22"/>
+      <c r="A65" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="B65" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C65" s="20"/>
+      <c r="D65" s="20"/>
+      <c r="E65" s="20"/>
+      <c r="F65" s="20"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="B66" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="C66" s="22"/>
-      <c r="D66" s="22"/>
-      <c r="E66" s="22"/>
-      <c r="F66" s="22"/>
+      <c r="A66" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="B66" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="23" t="s">
+      <c r="A67" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B67" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="B67" s="22" t="s">
-        <v>111</v>
-      </c>
-      <c r="C67" s="22"/>
-      <c r="D67" s="22"/>
-      <c r="E67" s="22"/>
-      <c r="F67" s="22"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="B69" s="24"/>
-      <c r="C69" s="24"/>
-      <c r="D69" s="24"/>
-      <c r="E69" s="24"/>
-      <c r="F69" s="24"/>
+      <c r="C67" s="20"/>
+      <c r="D67" s="20"/>
+      <c r="E67" s="20"/>
+      <c r="F67" s="20"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B68" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="C68" s="24"/>
+      <c r="D68" s="24"/>
+      <c r="E68" s="24"/>
+      <c r="F68" s="24"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="B69" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="C69" s="25"/>
+      <c r="D69" s="25"/>
+      <c r="E69" s="25"/>
+      <c r="F69" s="25"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="B70" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="C70" s="22"/>
-      <c r="D70" s="22"/>
-      <c r="E70" s="22"/>
-      <c r="F70" s="22"/>
+      <c r="B70" s="26"/>
+      <c r="C70" s="26"/>
+      <c r="D70" s="26"/>
+      <c r="E70" s="26"/>
+      <c r="F70" s="26"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="B71" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="C71" s="22"/>
-      <c r="D71" s="22"/>
-      <c r="E71" s="22"/>
-      <c r="F71" s="22"/>
+      <c r="A71" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="B71" s="24"/>
+      <c r="C71" s="24"/>
+      <c r="D71" s="24"/>
+      <c r="E71" s="24"/>
+      <c r="F71" s="24"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="B72" s="22" t="s">
-        <v>118</v>
-      </c>
-      <c r="C72" s="22"/>
-      <c r="D72" s="22"/>
-      <c r="E72" s="22"/>
-      <c r="F72" s="22"/>
+      <c r="A72" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="B72" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="C72" s="20"/>
+      <c r="D72" s="20"/>
+      <c r="E72" s="20"/>
+      <c r="F72" s="20"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="B73" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="C73" s="22"/>
-      <c r="D73" s="22"/>
-      <c r="E73" s="22"/>
-      <c r="F73" s="22"/>
-    </row>
-    <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="B74" s="22" t="s">
-        <v>122</v>
-      </c>
-      <c r="C74" s="22"/>
-      <c r="D74" s="22"/>
-      <c r="E74" s="22"/>
-      <c r="F74" s="22"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="24" t="s">
+      <c r="A73" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="B76" s="24"/>
-      <c r="C76" s="24"/>
-      <c r="D76" s="24"/>
-      <c r="E76" s="24"/>
-      <c r="F76" s="24"/>
-    </row>
-    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="15" t="s">
+      <c r="B73" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="B77" s="25" t="s">
+      <c r="C73" s="20"/>
+      <c r="D73" s="20"/>
+      <c r="E73" s="20"/>
+      <c r="F73" s="20"/>
+    </row>
+    <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="C77" s="25"/>
-      <c r="D77" s="25"/>
-      <c r="E77" s="25"/>
-      <c r="F77" s="25"/>
+      <c r="B74" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="C74" s="20"/>
+      <c r="D74" s="20"/>
+      <c r="E74" s="20"/>
+      <c r="F74" s="20"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="B75" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="C75" s="24"/>
+      <c r="D75" s="24"/>
+      <c r="E75" s="24"/>
+      <c r="F75" s="24"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="B76" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="C76" s="25"/>
+      <c r="D76" s="25"/>
+      <c r="E76" s="25"/>
+      <c r="F76" s="25"/>
+    </row>
+    <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B77" s="26"/>
+      <c r="C77" s="26"/>
+      <c r="D77" s="26"/>
+      <c r="E77" s="26"/>
+      <c r="F77" s="26"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="B78" s="25" t="s">
-        <v>127</v>
-      </c>
-      <c r="C78" s="25"/>
-      <c r="D78" s="25"/>
-      <c r="E78" s="25"/>
-      <c r="F78" s="25"/>
+      <c r="A78" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B78" s="24"/>
+      <c r="C78" s="24"/>
+      <c r="D78" s="24"/>
+      <c r="E78" s="24"/>
+      <c r="F78" s="24"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="B79" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="C79" s="25"/>
-      <c r="D79" s="25"/>
-      <c r="E79" s="25"/>
-      <c r="F79" s="25"/>
+      <c r="A79" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B79" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="C79" s="27"/>
+      <c r="D79" s="27"/>
+      <c r="E79" s="27"/>
+      <c r="F79" s="27"/>
+    </row>
+    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="B80" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="C80" s="24"/>
+      <c r="D80" s="24"/>
+      <c r="E80" s="24"/>
+      <c r="F80" s="24"/>
+    </row>
+    <row r="81" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="B81" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="C81" s="24"/>
+      <c r="D81" s="24"/>
+      <c r="E81" s="24"/>
+      <c r="F81" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="68">
@@ -4101,26 +4010,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>134</v>
+      <c r="A3" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B4" s="6" t="n">
         <v>0</v>
@@ -4135,7 +4044,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="B5" s="6" t="n">
         <v>0</v>
@@ -4149,8 +4058,8 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="27" t="s">
-        <v>137</v>
+      <c r="A6" s="17" t="s">
+        <v>145</v>
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">SUM(B4:B5)</f>
@@ -4167,18 +4076,18 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="26" t="s">
-        <v>139</v>
-      </c>
-      <c r="B10" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>141</v>
+      <c r="A10" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -4206,30 +4115,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>143</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>144</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>145</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>146</v>
-      </c>
-      <c r="E3" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="F3" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="G3" s="26" t="s">
-        <v>149</v>
+      <c r="A3" s="29" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>154</v>
+      </c>
+      <c r="E3" s="29" t="s">
+        <v>155</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>156</v>
+      </c>
+      <c r="G3" s="29" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -4260,23 +4169,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>151</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>152</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="E3" s="26" t="s">
+      <c r="A3" s="29" t="s">
+        <v>159</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E3" s="29" t="s">
         <v>39</v>
       </c>
     </row>
@@ -4306,41 +4215,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B3" s="26" t="s">
+      <c r="A3" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="C3" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="C3" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="E3" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="F3" s="26" t="s">
-        <v>156</v>
-      </c>
-      <c r="G3" s="26" t="s">
-        <v>157</v>
-      </c>
-      <c r="H3" s="26" t="s">
-        <v>158</v>
+      <c r="D3" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="G3" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="H3" s="29" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>0</v>
@@ -4358,17 +4267,17 @@
       <c r="G4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="28" t="n">
+      <c r="H4" s="30" t="n">
         <f aca="false">IFERROR(E4/D4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>0</v>
@@ -4386,17 +4295,17 @@
       <c r="G5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="28" t="n">
+      <c r="H5" s="30" t="n">
         <f aca="false">IFERROR(E5/D5,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>0</v>
@@ -4414,17 +4323,17 @@
       <c r="G6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="28" t="n">
+      <c r="H6" s="30" t="n">
         <f aca="false">IFERROR(E6/D6,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>0</v>
@@ -4442,17 +4351,17 @@
       <c r="G7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="28" t="n">
+      <c r="H7" s="30" t="n">
         <f aca="false">IFERROR(E7/D7,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>0</v>
@@ -4470,17 +4379,17 @@
       <c r="G8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="28" t="n">
+      <c r="H8" s="30" t="n">
         <f aca="false">IFERROR(E8/D8,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>0</v>
@@ -4498,14 +4407,14 @@
       <c r="G9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="28" t="n">
+      <c r="H9" s="30" t="n">
         <f aca="false">IFERROR(E9/D9,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="27" t="s">
-        <v>171</v>
+      <c r="A10" s="17" t="s">
+        <v>179</v>
       </c>
       <c r="C10" s="7" t="n">
         <f aca="false">SUM(C4:C9)</f>
@@ -4558,32 +4467,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>173</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>174</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>175</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="E3" s="26" t="s">
-        <v>156</v>
-      </c>
-      <c r="F3" s="26" t="s">
-        <v>158</v>
+      <c r="A3" s="29" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>182</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>183</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="E3" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>176</v>
+      <c r="A4" s="17" t="s">
+        <v>184</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>1</v>
@@ -4598,14 +4507,14 @@
         <f aca="false">C4-D4</f>
         <v>-2134.5</v>
       </c>
-      <c r="F4" s="28" t="n">
+      <c r="F4" s="30" t="n">
         <f aca="false">IFERROR(D4/C4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="s">
-        <v>177</v>
+      <c r="A5" s="17" t="s">
+        <v>185</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>0</v>
@@ -4620,14 +4529,14 @@
         <f aca="false">C5-D5</f>
         <v>0</v>
       </c>
-      <c r="F5" s="28" t="n">
+      <c r="F5" s="30" t="n">
         <f aca="false">IFERROR(D5/C5,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="27" t="s">
-        <v>178</v>
+      <c r="A6" s="17" t="s">
+        <v>186</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>3</v>
@@ -4642,14 +4551,14 @@
         <f aca="false">C6-D6</f>
         <v>-113811.85</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="30" t="n">
         <f aca="false">IFERROR(D6/C6,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="27" t="s">
-        <v>179</v>
+      <c r="A7" s="17" t="s">
+        <v>187</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>2</v>
@@ -4664,16 +4573,16 @@
         <f aca="false">C7-D7</f>
         <v>-1215.62</v>
       </c>
-      <c r="F7" s="28" t="n">
+      <c r="F7" s="30" t="n">
         <f aca="false">IFERROR(D7/C7,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="27" t="s">
-        <v>171</v>
-      </c>
-      <c r="B8" s="29" t="n">
+      <c r="A8" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="B8" s="31" t="n">
         <f aca="false">SUM(B4:B7)</f>
         <v>6</v>
       </c>
@@ -4722,43 +4631,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="30" t="s">
-        <v>181</v>
+      <c r="A2" s="32" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="E4" s="26" t="s">
-        <v>156</v>
-      </c>
-      <c r="F4" s="26" t="s">
-        <v>182</v>
-      </c>
-      <c r="G4" s="26" t="s">
+      <c r="A4" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="E4" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="F4" s="29" t="s">
+        <v>190</v>
+      </c>
+      <c r="G4" s="29" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>0</v>
@@ -4770,21 +4679,21 @@
         <f aca="false">C5-D5</f>
         <v>-2134.5</v>
       </c>
-      <c r="F5" s="28" t="n">
+      <c r="F5" s="30" t="n">
         <f aca="false">IFERROR((D5-C5)/C5,0)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="31" t="str">
+      <c r="G5" s="33" t="str">
         <f aca="false">IF(C5=0,"UNBUDGETED",IF(F5&gt;0.5,"CRITICAL",IF(F5&gt;0.1,"OVER",IF(F5&lt;-0.1,"UNDER","ON"))))</f>
         <v>UNBUDGETED</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>0</v>
@@ -4796,21 +4705,21 @@
         <f aca="false">C6-D6</f>
         <v>-106487.5</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="30" t="n">
         <f aca="false">IFERROR((D6-C6)/C6,0)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="31" t="str">
+      <c r="G6" s="33" t="str">
         <f aca="false">IF(C6=0,"UNBUDGETED",IF(F6&gt;0.5,"CRITICAL",IF(F6&gt;0.1,"OVER",IF(F6&lt;-0.1,"UNDER","ON"))))</f>
         <v>UNBUDGETED</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>0</v>
@@ -4822,21 +4731,21 @@
         <f aca="false">C7-D7</f>
         <v>-922.35</v>
       </c>
-      <c r="F7" s="28" t="n">
+      <c r="F7" s="30" t="n">
         <f aca="false">IFERROR((D7-C7)/C7,0)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="31" t="str">
+      <c r="G7" s="33" t="str">
         <f aca="false">IF(C7=0,"UNBUDGETED",IF(F7&gt;0.5,"CRITICAL",IF(F7&gt;0.1,"OVER",IF(F7&lt;-0.1,"UNDER","ON"))))</f>
         <v>UNBUDGETED</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>0</v>
@@ -4848,21 +4757,21 @@
         <f aca="false">C8-D8</f>
         <v>-6402</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="30" t="n">
         <f aca="false">IFERROR((D8-C8)/C8,0)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="31" t="str">
+      <c r="G8" s="33" t="str">
         <f aca="false">IF(C8=0,"UNBUDGETED",IF(F8&gt;0.5,"CRITICAL",IF(F8&gt;0.1,"OVER",IF(F8&lt;-0.1,"UNDER","ON"))))</f>
         <v>UNBUDGETED</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>0</v>
@@ -4874,21 +4783,21 @@
         <f aca="false">C9-D9</f>
         <v>-1052.32</v>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="30" t="n">
         <f aca="false">IFERROR((D9-C9)/C9,0)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="31" t="str">
+      <c r="G9" s="33" t="str">
         <f aca="false">IF(C9=0,"UNBUDGETED",IF(F9&gt;0.5,"CRITICAL",IF(F9&gt;0.1,"OVER",IF(F9&lt;-0.1,"UNDER","ON"))))</f>
         <v>UNBUDGETED</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>0</v>
@@ -4900,11 +4809,11 @@
         <f aca="false">C10-D10</f>
         <v>-163.3</v>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="30" t="n">
         <f aca="false">IFERROR((D10-C10)/C10,0)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="31" t="str">
+      <c r="G10" s="33" t="str">
         <f aca="false">IF(C10=0,"UNBUDGETED",IF(F10&gt;0.5,"CRITICAL",IF(F10&gt;0.1,"OVER",IF(F10&lt;-0.1,"UNDER","ON"))))</f>
         <v>UNBUDGETED</v>
       </c>
@@ -4936,26 +4845,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>184</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>185</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>186</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>187</v>
+      <c r="A3" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>193</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>194</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B4" s="6" t="n">
         <v>90628.75</v>
@@ -4963,14 +4872,14 @@
       <c r="C4" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="D4" s="28" t="n">
+      <c r="D4" s="30" t="n">
         <f aca="false">IFERROR(B4/SUM(B$4:B$6),0)</f>
         <v>0.925225949969935</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="B5" s="6" t="n">
         <v>6402</v>
@@ -4978,14 +4887,14 @@
       <c r="C5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="30" t="n">
         <f aca="false">IFERROR(B5/SUM(B$4:B$6),0)</f>
         <v>0.0653578089922626</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>922.35</v>
@@ -4993,20 +4902,20 @@
       <c r="C6" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="28" t="n">
+      <c r="D6" s="30" t="n">
         <f aca="false">IFERROR(B6/SUM(B$4:B$6),0)</f>
         <v>0.00941624103780279</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="27" t="s">
-        <v>191</v>
+      <c r="A7" s="17" t="s">
+        <v>199</v>
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">SUM(B4:B6)</f>
         <v>97953.1</v>
       </c>
-      <c r="C7" s="32" t="n">
+      <c r="C7" s="34" t="n">
         <f aca="false">SUM(C4:C6)</f>
         <v>12</v>
       </c>

</xml_diff>